<commit_message>
Complete warehouse audit decision guidance and worked examples
Carry a fictional inventory finding through correction, accountable action and
verification, and give the 3PL renewal example separate service, storage and
billing conclusions. Align the Excel, PDF and browser preview with those cases.

Explain audit criteria, reviewer responsibilities and escalation, and add a
cost/capacity commissioning example for directors. Make public printing visible
and preserve legacy section links while retaining the approved artwork and
subscription design.

Mark PDF assets as binary so required cross-reference whitespace is not treated
as source-code whitespace.
</commit_message>
<xml_diff>
--- a/public/files/warehouse-audit-working-pack.xlsx
+++ b/public/files/warehouse-audit-working-pack.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R31b0e689c8fe41bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope and criteria" sheetId="2" r:id="R74207fbe94e24b1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist and evidence" sheetId="3" r:id="Rf2c577f1d9374a9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings and actions" sheetId="4" r:id="Rc449a8c5802741db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Management review" sheetId="5" r:id="R05e228dcce544114"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worked examples" sheetId="6" r:id="R99820d8006094f94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R008e8739509946fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope and criteria" sheetId="2" r:id="Rf878174ba3d5483a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist and evidence" sheetId="3" r:id="Rac38dfd486924671"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings and actions" sheetId="4" r:id="Rf7e4a5b2f9eb42f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Management review" sheetId="5" r:id="R1ea0b476166e4b5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worked examples" sheetId="6" r:id="Re7f550447ad34585"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1027,7 +1027,7 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="R48c239dc96144bb1"/>
+    <tablePart r:id="Rf5a8a04dfafb4067"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1628,9 +1628,9 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cc7513b8fc7430b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6fbfdd33eba4f6c"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a4e19949f374157"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10aaa44b26664f7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R231fc6554b6d4f79"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33a78978e3db459a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3470,8 +3470,8 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
-    <tablePart r:id="Rd20b3f6a005d41d6"/>
-    <tablePart r:id="R8d18320d3b7f4610"/>
+    <tablePart r:id="Rf098649c98d74f22"/>
+    <tablePart r:id="R7a8228667720427c"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4836,9 +4836,9 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ae7a6b90c35430a"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1760d98085fc4cef"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fae9c090dd44601"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R495a68d7b72e45f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66ac0f93a5974ad8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f25e9d2faa34f9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5130,8 +5130,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red59d1b753ff4e59"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e0902d83287447b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f7afc5d06c34a87"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76cae2a65fd64d5c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5181,7 +5181,7 @@
         <x:v>Example status</x:v>
       </x:c>
       <x:c r="B7" s="29" t="str">
-        <x:v>Fictional worked example — investigation remains open</x:v>
+        <x:v>Fictional worked example — correction and limited verification recorded</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
@@ -5189,7 +5189,7 @@
         <x:v>Purpose</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>Show how a confirmed difference can be recorded without inventing its cause or treating a balance adjustment as closure.</x:v>
+        <x:v>Follow one evidenced stock difference through correction, a process action and verification. Keep older recurrences unresolved.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -5209,7 +5209,7 @@
         <x:v>Site or area alias</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>Example bin A-01</x:v>
+        <x:v>Example bin A01</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="45" customHeight="1">
@@ -5217,7 +5217,7 @@
         <x:v>Review date or period</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>Comparison time and review dates not yet recorded.</x:v>
+        <x:v>Count comparison: 6 October 2026, 09:00. Follow-up: 9 October 2026, 15:00.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="45" customHeight="1">
@@ -5225,7 +5225,7 @@
         <x:v>Operating conditions</x:v>
       </x:c>
       <x:c r="B13" s="7" t="str">
-        <x:v>Movement timing and unit history remain to be reconciled.</x:v>
+        <x:v>One unit dispatched on 5 October at 16:40. Its stock issue was still pending at the count.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="45" customHeight="1">
@@ -5233,7 +5233,7 @@
         <x:v>Coverage and sample</x:v>
       </x:c>
       <x:c r="B14" s="7" t="str">
-        <x:v>SKU-104 in bin A-01; count, recount and selected receipt/issue records. Linked checks INV01, INV02 and INV03.</x:v>
+        <x:v>SKU104, bin A01. Count/recount and transaction trail; follow-up covers 20 dispatches on 7–9 October across three shifts. Checks INV01–03.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="45" customHeight="1">
@@ -5241,7 +5241,7 @@
         <x:v>Exclusions and limits</x:v>
       </x:c>
       <x:c r="B15" s="7" t="str">
-        <x:v>This one-item example does not establish the condition of the whole inventory.</x:v>
+        <x:v>Older discrepancies remain unexplained. This item and limited follow-up sample do not establish performance across all stock or shifts.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="45" customHeight="1">
@@ -5249,7 +5249,7 @@
         <x:v>Criteria and versions</x:v>
       </x:c>
       <x:c r="B16" s="7" t="str">
-        <x:v>Site inventory procedure identified; version, comparison boundary and applicable steps not yet recorded.</x:v>
+        <x:v>Fictional procedure INV04 v3: post each stock issue before dispatch. Compare the same item, unit, location and time.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="45" customHeight="1">
@@ -5257,7 +5257,7 @@
         <x:v>Reviewer and evidence providers</x:v>
       </x:c>
       <x:c r="B17" s="7" t="str">
-        <x:v>Reviewer and any required independent verification not yet assigned.</x:v>
+        <x:v>Inventory lead traces C104, RC104, S104, P418, D418 and Q418. Warehouse manager verifies the follow-up in V104.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="45" customHeight="1">
@@ -5265,7 +5265,7 @@
         <x:v>Action responsibilities</x:v>
       </x:c>
       <x:c r="B18" s="7" t="str">
-        <x:v>Inventory lead, working with the process/system owner.</x:v>
+        <x:v>Inventory lead owns the handover change and pending-issue review, due 6 October 2026, 17:00.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="45" customHeight="1">
@@ -5273,7 +5273,7 @@
         <x:v>Decision owner</x:v>
       </x:c>
       <x:c r="B19" s="7" t="str">
-        <x:v>Adjustment or resource authority to be established under the site's procedure.</x:v>
+        <x:v>Inventory manager authorises posting the one missing issue on 6 October 2026, 11:00.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
@@ -5323,7 +5323,7 @@
         <x:v>Criterion / reference</x:v>
       </x:c>
       <x:c r="B26" s="7" t="str">
-        <x:v>Site inventory procedure. Version and effective comparison criteria not yet recorded.</x:v>
+        <x:v>Fictional site procedure INV04 v3 requires each stock issue to be posted before dispatch.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="60" customHeight="1">
@@ -5331,7 +5331,7 @@
         <x:v>Observation</x:v>
       </x:c>
       <x:c r="B27" s="7" t="str">
-        <x:v>The physical count for SKU-104 in bin A-01 is 11 units; the inventory record shows 12. A recount confirms 11.</x:v>
+        <x:v>At 09:00 on 6 October 2026, C104 and independent recount RC104 show 11 each of SKU104 in bin A01. Snapshot S104 shows 12.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
@@ -5339,7 +5339,7 @@
         <x:v>Evidence obtained</x:v>
       </x:c>
       <x:c r="B28" s="7" t="str">
-        <x:v>Count note, recount, stock-record comparison and references to selected receipt/issue records in this fictional case.</x:v>
+        <x:v>P418 and D418 record one unit leaving on 5 October at 16:40. Q418 shows that issue still pending at the count.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="60" customHeight="1">
@@ -5347,7 +5347,7 @@
         <x:v>Evidence still needed</x:v>
       </x:c>
       <x:c r="B29" s="7" t="str">
-        <x:v>Reconcile receipt/issue timing, the record snapshot and unit/pack definitions at the comparison point.</x:v>
+        <x:v>Investigate the separate older recurrences. This transaction trail does not explain those earlier differences.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="60" customHeight="1">
@@ -5355,7 +5355,7 @@
         <x:v>Uncertainty</x:v>
       </x:c>
       <x:c r="B30" s="7" t="str">
-        <x:v>The difference is confirmed. Its cause, full transaction boundary and required action remain unresolved.</x:v>
+        <x:v>The unposted issue explains this one-unit difference. Why it remained pending and the causes of older recurrences are not established.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
@@ -5363,7 +5363,7 @@
         <x:v>Possible cause (hypothesis)</x:v>
       </x:c>
       <x:c r="B31" s="7" t="str">
-        <x:v>Hypothesis only: unit-of-measure or transaction-timing issue. Neither is established.</x:v>
+        <x:v>Evidence confirms one unposted issue. It does not establish fraud or a root cause for all recurring discrepancies.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="60" customHeight="1">
@@ -5371,7 +5371,7 @@
         <x:v>Next action</x:v>
       </x:c>
       <x:c r="B32" s="7" t="str">
-        <x:v>Compare the receipt/issue trail and unit definitions with the process/system owner. Retain the explanation supported by evidence. Handle any balance adjustment separately under the authorised process.</x:v>
+        <x:v>Post the single missing issue with approval. Give handover a named owner and review pending issues before release. Retain older cases for investigation.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
@@ -5379,7 +5379,7 @@
         <x:v>Action type</x:v>
       </x:c>
       <x:c r="B33" s="7" t="str">
-        <x:v>Investigation</x:v>
+        <x:v>Authorised correction, corrective action and verification</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
@@ -5395,7 +5395,7 @@
         <x:v>Target date</x:v>
       </x:c>
       <x:c r="B35" s="7" t="str">
-        <x:v>Not yet agreed</x:v>
+        <x:v>6 October 2026, 17:00, for handover ownership and the pending-issue review.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
@@ -5403,7 +5403,7 @@
         <x:v>Urgency</x:v>
       </x:c>
       <x:c r="B36" s="7" t="str">
-        <x:v>Not assessed</x:v>
+        <x:v>Inventory manager requires the record correction and control change on 6 October. No wider urgency conclusion is made.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
@@ -5411,7 +5411,7 @@
         <x:v>Work state</x:v>
       </x:c>
       <x:c r="B37" s="7" t="str">
-        <x:v>Open — investigation not completed</x:v>
+        <x:v>6 October: manager approves posting at 11:00. Records then show 11. H104 records named handover ownership and pre-release pending-issue review in use by 17:00.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="60" customHeight="1">
@@ -5419,7 +5419,7 @@
         <x:v>Verification method</x:v>
       </x:c>
       <x:c r="B38" s="7" t="str">
-        <x:v>After an evidenced action is chosen, examine subsequent relevant transactions and counts against the agreed criterion. Define the sample and timing before verification.</x:v>
+        <x:v>V104: compare 20 dispatches on 7–9 October across three shifts with INV04 v3. Check issue posting before release and recount the selected bin.</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
@@ -5427,7 +5427,7 @@
         <x:v>Verification owner</x:v>
       </x:c>
       <x:c r="B39" s="7" t="str">
-        <x:v>Not yet assigned</x:v>
+        <x:v>Warehouse manager</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
@@ -5435,7 +5435,7 @@
         <x:v>Verification date</x:v>
       </x:c>
       <x:c r="B40" s="7" t="str">
-        <x:v>Not yet agreed</x:v>
+        <x:v>9 October 2026, 15:00</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
@@ -5443,7 +5443,7 @@
         <x:v>Verification result</x:v>
       </x:c>
       <x:c r="B41" s="7" t="str">
-        <x:v>Pending — no effectiveness conclusion</x:v>
+        <x:v>Effective in the examined sample: all 20 issues posted before release and the selected bin matches. Older recurrences remain unresolved.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
@@ -5451,7 +5451,7 @@
         <x:v>Decision / resources needed</x:v>
       </x:c>
       <x:c r="B42" s="7" t="str">
-        <x:v>Establish adjustment authority and any process/system decision once the evidence is reviewed.</x:v>
+        <x:v>The manager approves posting the one missing issue. No additional balance adjustment is made, which would double-count the correction.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
@@ -5459,7 +5459,7 @@
         <x:v>Decision owner</x:v>
       </x:c>
       <x:c r="B43" s="7" t="str">
-        <x:v>Not yet established</x:v>
+        <x:v>Inventory manager for correction authority; inventory lead for the process action and older-case investigation.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="30" customHeight="1">
@@ -5471,7 +5471,7 @@
         <x:v>Management note</x:v>
       </x:c>
       <x:c r="B45" s="7" t="str">
-        <x:v>Keep the one-unit difference, uncertain explanation and missing verification assignment visible. The case does not establish a missed pick, loss or successful fix.</x:v>
+        <x:v>Close this recorded correction and sampled follow-up. Keep older recurrences open. V104 supports the result only for the examined sample.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="30" customHeight="1">
@@ -5501,7 +5501,7 @@
         <x:v>Purpose</x:v>
       </x:c>
       <x:c r="B50" s="7" t="str">
-        <x:v>Bring service, storage and billing evidence to one decision while retaining separate criteria, owners and unanswered questions.</x:v>
+        <x:v>Bring service, storage and billing evidence to a renewal review. Show a verified credit alongside service and storage questions that remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="30" customHeight="1">
@@ -5529,7 +5529,7 @@
         <x:v>Review date or period</x:v>
       </x:c>
       <x:c r="B54" s="7" t="str">
-        <x:v>Renewal review period, shipment sample and billed period not yet agreed.</x:v>
+        <x:v>Review as at 8 October 2026. Service and billed-activity period: 1–7 October 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="45" customHeight="1">
@@ -5537,7 +5537,7 @@
         <x:v>Operating conditions</x:v>
       </x:c>
       <x:c r="B55" s="7" t="str">
-        <x:v>Workload, staffing and exception context to be obtained for selected shipments.</x:v>
+        <x:v>Investigate the four late orders. Product acceptability remains unresolved because the 2 October condition record is missing.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="45" customHeight="1">
@@ -5545,7 +5545,7 @@
         <x:v>Coverage and sample</x:v>
       </x:c>
       <x:c r="B56" s="7" t="str">
-        <x:v>Selected late dispatches, goods affected by the storage concern and disputed invoice lines. Linked checks FLOW03, FLOW04, GOODS02, GOODS04, CONTROL03 and CONTROL04.</x:v>
+        <x:v>12 orders, goods affected by the 2 October record gap and one invoice line for 120 pallet-days. Checks FLOW03–04, GOODS02, GOODS04 and CONTROL03–04.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="45" customHeight="1">
@@ -5553,7 +5553,7 @@
         <x:v>Exclusions and limits</x:v>
       </x:c>
       <x:c r="B57" s="7" t="str">
-        <x:v>This review has not established all provider qualifications or every product, legal or commercial requirement.</x:v>
+        <x:v>No conclusion on all provider qualifications or all shipments. Fictional invoice amounts exclude VAT and other lines.</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="45" customHeight="1">
@@ -5561,7 +5561,7 @@
         <x:v>Criteria and versions</x:v>
       </x:c>
       <x:c r="B58" s="7" t="str">
-        <x:v>Dispatch commitment, goods/customer storage requirement and applicable contract/rate version remain to be obtained and assigned to the relevant issue.</x:v>
+        <x:v>SLA12 v2: orders ready for 17:00 dispatch. CS2 v2: customer dry-storage requirement. Signed rate v2: £1.50 per pallet-day from 1 October.</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="45" customHeight="1">
@@ -5569,7 +5569,7 @@
         <x:v>Reviewer and evidence providers</x:v>
       </x:c>
       <x:c r="B59" s="7" t="str">
-        <x:v>Service, product/quality and commercial/finance owners provide evidence. Review responsibilities and any specialist assessment to be agreed.</x:v>
+        <x:v>Service lead checks order/staging/handover records. Quality lead assesses the record gap. Commercial lead reconciles billing; finance controller checks CN82.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="45" customHeight="1">
@@ -5577,7 +5577,7 @@
         <x:v>Action responsibilities</x:v>
       </x:c>
       <x:c r="B60" s="7" t="str">
-        <x:v>A separate responsible owner for each issue.</x:v>
+        <x:v>Service lead: report by 10 October. Quality lead: assessment by 9 October. Commercial lead: credit and contract timetable/options.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="45" customHeight="1">
@@ -5585,7 +5585,7 @@
         <x:v>Decision owner</x:v>
       </x:c>
       <x:c r="B61" s="7" t="str">
-        <x:v>Logistics director for renewal; other approval authorities to be established where required.</x:v>
+        <x:v>Logistics director requests the service plan and quality assessment on 8 October before a final renewal decision.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="30" customHeight="1">
@@ -5627,7 +5627,7 @@
         <x:v>Review status</x:v>
       </x:c>
       <x:c r="B67" s="7" t="str">
-        <x:v>Inconclusive or conflicting evidence</x:v>
+        <x:v>Concern found</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="42" customHeight="1">
@@ -5635,7 +5635,7 @@
         <x:v>Criterion / reference</x:v>
       </x:c>
       <x:c r="B68" s="7" t="str">
-        <x:v>Agreed dispatch commitment and relevant agreement version not yet attached.</x:v>
+        <x:v>Fictional SLA12 v2 requires the selected orders to be ready for 17:00 dispatch.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="60" customHeight="1">
@@ -5643,7 +5643,7 @@
         <x:v>Observation</x:v>
       </x:c>
       <x:c r="B69" s="7" t="str">
-        <x:v>Recent dispatches are reported late. The selected shipment records have not yet been compared with the agreed commitment.</x:v>
+        <x:v>Four of 12 selected orders from 1–7 October 2026 were late against the agreed dispatch-readiness commitment.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="42" customHeight="1">
@@ -5651,7 +5651,7 @@
         <x:v>Evidence obtained</x:v>
       </x:c>
       <x:c r="B70" s="7" t="str">
-        <x:v>Reported service concern in this fictional case; supporting timestamps not yet attached.</x:v>
+        <x:v>Order, staging and handover records for the 12 orders establish the four exceptions against SLA12 v2.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="60" customHeight="1">
@@ -5659,7 +5659,7 @@
         <x:v>Evidence still needed</x:v>
       </x:c>
       <x:c r="B71" s="7" t="str">
-        <x:v>Agreed commitment, order-release and actual dispatch timestamps, workload, staffing and exception records for the selected shipments.</x:v>
+        <x:v>Service lead to examine staffing, workload, queues and exceptions around the four late orders and propose a supported service plan.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="60" customHeight="1">
@@ -5667,7 +5667,7 @@
         <x:v>Uncertainty</x:v>
       </x:c>
       <x:c r="B72" s="7" t="str">
-        <x:v>Extent, contractual significance and reason for the delays remain unconfirmed.</x:v>
+        <x:v>The four exceptions are established within this sample. Their cause and wider service performance remain under investigation.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="42" customHeight="1">
@@ -5675,7 +5675,7 @@
         <x:v>Possible cause (hypothesis)</x:v>
       </x:c>
       <x:c r="B73" s="7" t="str">
-        <x:v>Not established</x:v>
+        <x:v>Not yet established. The observed lateness does not identify a particular operating cause.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="60" customHeight="1">
@@ -5683,7 +5683,7 @@
         <x:v>Next action</x:v>
       </x:c>
       <x:c r="B74" s="7" t="str">
-        <x:v>Obtain and compare the selected shipment records with the commitment; identify the constraint supported by the evidence.</x:v>
+        <x:v>Service lead reports the evidence, remaining cause questions and proposed plan to the director by 10 October 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="42" customHeight="1">
@@ -5699,7 +5699,7 @@
         <x:v>Responsible owner</x:v>
       </x:c>
       <x:c r="B76" s="7" t="str">
-        <x:v>Service owner</x:v>
+        <x:v>Service lead</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="42" customHeight="1">
@@ -5707,7 +5707,7 @@
         <x:v>Target date</x:v>
       </x:c>
       <x:c r="B77" s="7" t="str">
-        <x:v>Not yet agreed</x:v>
+        <x:v>10 October 2026</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="42" customHeight="1">
@@ -5715,7 +5715,7 @@
         <x:v>Urgency</x:v>
       </x:c>
       <x:c r="B78" s="7" t="str">
-        <x:v>Not assessed</x:v>
+        <x:v>Director requires the service plan before the final renewal decision.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="42" customHeight="1">
@@ -5723,7 +5723,7 @@
         <x:v>Work state</x:v>
       </x:c>
       <x:c r="B79" s="7" t="str">
-        <x:v>Open — evidence requested</x:v>
+        <x:v>Open as at 8 October: investigation and service plan due 10 October.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="60" customHeight="1">
@@ -5731,7 +5731,7 @@
         <x:v>Verification method</x:v>
       </x:c>
       <x:c r="B80" s="7" t="str">
-        <x:v>Once an action and service criterion are agreed, compare later relevant shipment performance and exception records. Verification period not yet established.</x:v>
+        <x:v>After agreeing the plan, warehouse manager checks later order/staging/handover records against SLA12 v2. Agree coverage and timing with the plan.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="42" customHeight="1">
@@ -5739,7 +5739,7 @@
         <x:v>Verification owner</x:v>
       </x:c>
       <x:c r="B81" s="7" t="str">
-        <x:v>Not yet assigned</x:v>
+        <x:v>Warehouse manager</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="42" customHeight="1">
@@ -5747,7 +5747,7 @@
         <x:v>Verification date</x:v>
       </x:c>
       <x:c r="B82" s="7" t="str">
-        <x:v>Not yet agreed</x:v>
+        <x:v>To be agreed after the service plan</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="42" customHeight="1">
@@ -5763,7 +5763,7 @@
         <x:v>Decision / resources needed</x:v>
       </x:c>
       <x:c r="B84" s="7" t="str">
-        <x:v>Consider any evidenced resource or service condition as part of renewal.</x:v>
+        <x:v>Director requests a service plan before final renewal. Commercial lead checks the contract timetable and available options.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="42" customHeight="1">
@@ -5821,7 +5821,7 @@
         <x:v>Criterion / reference</x:v>
       </x:c>
       <x:c r="B92" s="7" t="str">
-        <x:v>Actual product/customer storage requirement and its applicable version not yet established.</x:v>
+        <x:v>Fictional customer requirement CS2 v2 specifies dry storage for the affected goods.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="60" customHeight="1">
@@ -5829,7 +5829,7 @@
         <x:v>Observation</x:v>
       </x:c>
       <x:c r="B93" s="7" t="str">
-        <x:v>A customer has raised a storage concern. The affected goods, location and acceptability have not yet been established.</x:v>
+        <x:v>The 2 October 2026 condition record is missing for the affected goods. The available evidence cannot establish acceptability.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="42" customHeight="1">
@@ -5837,7 +5837,7 @@
         <x:v>Evidence obtained</x:v>
       </x:c>
       <x:c r="B94" s="7" t="str">
-        <x:v>Reported customer concern in this fictional case; supporting condition records not yet attached.</x:v>
+        <x:v>CS2 v2 and the condition-record review identify the specific 2 October gap.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="60" customHeight="1">
@@ -5845,7 +5845,7 @@
         <x:v>Evidence still needed</x:v>
       </x:c>
       <x:c r="B95" s="7" t="str">
-        <x:v>Affected goods/location, applicable storage requirement, monitoring records, reported exception and competent assessment of acceptability.</x:v>
+        <x:v>Quality lead to assess the affected goods, remaining condition evidence and any action needed under CS2 v2.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="60" customHeight="1">
@@ -5853,7 +5853,7 @@
         <x:v>Uncertainty</x:v>
       </x:c>
       <x:c r="B96" s="7" t="str">
-        <x:v>The concern does not establish product condition, a breached requirement or the required disposition.</x:v>
+        <x:v>Missing evidence does not establish acceptable or unacceptable goods. Product acceptability and any disposition remain for quality assessment.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="42" customHeight="1">
@@ -5869,7 +5869,7 @@
         <x:v>Next action</x:v>
       </x:c>
       <x:c r="B98" s="7" t="str">
-        <x:v>Establish the applicable requirement, assess the affected goods and determine any action and verification needed.</x:v>
+        <x:v>Quality lead assesses the affected goods and evidence gap under CS2 v2 and reports to the director by 9 October 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="42" customHeight="1">
@@ -5885,7 +5885,7 @@
         <x:v>Responsible owner</x:v>
       </x:c>
       <x:c r="B100" s="7" t="str">
-        <x:v>Product/quality owner</x:v>
+        <x:v>Quality lead</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="42" customHeight="1">
@@ -5893,7 +5893,7 @@
         <x:v>Target date</x:v>
       </x:c>
       <x:c r="B101" s="7" t="str">
-        <x:v>Not yet agreed</x:v>
+        <x:v>9 October 2026</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="42" customHeight="1">
@@ -5901,7 +5901,7 @@
         <x:v>Urgency</x:v>
       </x:c>
       <x:c r="B102" s="7" t="str">
-        <x:v>Not assessed</x:v>
+        <x:v>Director requires the quality assessment before final renewal. Quality lead determines any response needed for the goods.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="42" customHeight="1">
@@ -5909,7 +5909,7 @@
         <x:v>Work state</x:v>
       </x:c>
       <x:c r="B103" s="7" t="str">
-        <x:v>Open — requirement and assessment outstanding</x:v>
+        <x:v>Open as at 8 October: quality assessment due 9 October.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="60" customHeight="1">
@@ -5917,7 +5917,7 @@
         <x:v>Verification method</x:v>
       </x:c>
       <x:c r="B104" s="7" t="str">
-        <x:v>Define the evidence needed to verify the chosen action against the actual storage requirement; method remains to be agreed by the responsible assessor.</x:v>
+        <x:v>Quality lead defines any required action and evidence of its effectiveness against CS2 v2 after assessing the affected goods.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="42" customHeight="1">
@@ -5925,7 +5925,7 @@
         <x:v>Verification owner</x:v>
       </x:c>
       <x:c r="B105" s="7" t="str">
-        <x:v>Not yet assigned</x:v>
+        <x:v>Quality lead; any additional assessor to be identified through the assessment.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="42" customHeight="1">
@@ -5933,7 +5933,7 @@
         <x:v>Verification date</x:v>
       </x:c>
       <x:c r="B106" s="7" t="str">
-        <x:v>Not yet agreed</x:v>
+        <x:v>To be agreed after the quality assessment</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="42" customHeight="1">
@@ -5949,7 +5949,7 @@
         <x:v>Decision / resources needed</x:v>
       </x:c>
       <x:c r="B108" s="7" t="str">
-        <x:v>Bring the assessment, required action and remaining uncertainty into the renewal review.</x:v>
+        <x:v>Director requests the quality assessment before final renewal. Keep the condition-record gap and any product decision visible.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="42" customHeight="1">
@@ -5957,7 +5957,7 @@
         <x:v>Decision owner</x:v>
       </x:c>
       <x:c r="B109" s="7" t="str">
-        <x:v>Logistics director; product disposition authority not yet established</x:v>
+        <x:v>Logistics director for renewal; quality lead to establish the required product decision and authority.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="30" customHeight="1">
@@ -5999,7 +5999,7 @@
         <x:v>Review status</x:v>
       </x:c>
       <x:c r="B115" s="7" t="str">
-        <x:v>Inconclusive or conflicting evidence</x:v>
+        <x:v>Concern found</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="42" customHeight="1">
@@ -6007,7 +6007,7 @@
         <x:v>Criterion / reference</x:v>
       </x:c>
       <x:c r="B116" s="7" t="str">
-        <x:v>Applicable contract/rate version, charging basis and billed period not yet attached.</x:v>
+        <x:v>Signed fictional rate v2, effective 1 October 2026: £1.50 per pallet-day for the same unit and billed period.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="60" customHeight="1">
@@ -6015,7 +6015,7 @@
         <x:v>Observation</x:v>
       </x:c>
       <x:c r="B117" s="7" t="str">
-        <x:v>Some invoice charges are disputed. The relevant invoice lines have not yet been reconciled to the agreement and activity records.</x:v>
+        <x:v>Invoice bills 120 pallet-days at £2 = £240. Activity records confirm 120. Rate v2 gives 120 × £1.50 = £180, a £60 difference.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="42" customHeight="1">
@@ -6023,7 +6023,7 @@
         <x:v>Evidence obtained</x:v>
       </x:c>
       <x:c r="B118" s="7" t="str">
-        <x:v>Reported billing dispute in this fictional case; selected invoice and activity references not yet attached.</x:v>
+        <x:v>Invoice line, matching 1–7 October activity records, signed rate v2 and obsolete v1 identify the rate error. CN82 records the agreed £60 credit.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="60" customHeight="1">
@@ -6031,7 +6031,7 @@
         <x:v>Evidence still needed</x:v>
       </x:c>
       <x:c r="B119" s="7" t="str">
-        <x:v>Contract/rate version, invoice lines, charging units, movement/storage/service records for the billed period and documented exceptions.</x:v>
+        <x:v>None for this reconciled line and credit. Other invoice lines and VAT are outside the example.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="60" customHeight="1">
@@ -6039,7 +6039,7 @@
         <x:v>Uncertainty</x:v>
       </x:c>
       <x:c r="B120" s="7" t="str">
-        <x:v>Interpretation, entitlement and any adjustment remain unresolved. No saving has been established.</x:v>
+        <x:v>The fictional calculation excludes VAT and other lines. It establishes no external contract entitlement or wider ROI.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="42" customHeight="1">
@@ -6047,7 +6047,7 @@
         <x:v>Possible cause (hypothesis)</x:v>
       </x:c>
       <x:c r="B121" s="7" t="str">
-        <x:v>Not established</x:v>
+        <x:v>Obsolete v1 rate was used instead of signed v2. The source of that rate-selection error is not established.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="60" customHeight="1">
@@ -6055,7 +6055,7 @@
         <x:v>Next action</x:v>
       </x:c>
       <x:c r="B122" s="7" t="str">
-        <x:v>Reconcile the selected invoice lines and charging units with the agreement and activity evidence; record any interpretation needing a decision.</x:v>
+        <x:v>Commercial lead agrees CN82 for £60 on 8 October. Finance controller checks the credit and net £180 on the same day.</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="42" customHeight="1">
@@ -6063,7 +6063,7 @@
         <x:v>Action type</x:v>
       </x:c>
       <x:c r="B123" s="7" t="str">
-        <x:v>Investigation</x:v>
+        <x:v>Agreed billing correction and verification</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="42" customHeight="1">
@@ -6071,7 +6071,7 @@
         <x:v>Responsible owner</x:v>
       </x:c>
       <x:c r="B124" s="7" t="str">
-        <x:v>Commercial/finance owner</x:v>
+        <x:v>Commercial lead</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="42" customHeight="1">
@@ -6079,7 +6079,7 @@
         <x:v>Target date</x:v>
       </x:c>
       <x:c r="B125" s="7" t="str">
-        <x:v>Not yet agreed</x:v>
+        <x:v>8 October 2026</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="42" customHeight="1">
@@ -6087,7 +6087,7 @@
         <x:v>Urgency</x:v>
       </x:c>
       <x:c r="B126" s="7" t="str">
-        <x:v>Not assessed</x:v>
+        <x:v>Resolve this line within the 8 October commercial review. Service and storage questions remain separate.</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="42" customHeight="1">
@@ -6095,7 +6095,7 @@
         <x:v>Work state</x:v>
       </x:c>
       <x:c r="B127" s="7" t="str">
-        <x:v>Open — reconciliation outstanding</x:v>
+        <x:v>8 October 2026: commercial lead agrees £60 credit CN82. Finance controller verifies the resulting £180 net charge.</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="60" customHeight="1">
@@ -6103,7 +6103,7 @@
         <x:v>Verification method</x:v>
       </x:c>
       <x:c r="B128" s="7" t="str">
-        <x:v>Check any agreed resolution against the reconciled activity and resulting invoice or credit record. Requirements and reviewer remain to be agreed.</x:v>
+        <x:v>Reconcile the 120 pallet-days to signed rate v2 and check £240 invoice less £60 credit CN82 equals £180.</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="42" customHeight="1">
@@ -6111,7 +6111,7 @@
         <x:v>Verification owner</x:v>
       </x:c>
       <x:c r="B129" s="7" t="str">
-        <x:v>Not yet assigned</x:v>
+        <x:v>Finance controller</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="42" customHeight="1">
@@ -6119,7 +6119,7 @@
         <x:v>Verification date</x:v>
       </x:c>
       <x:c r="B130" s="7" t="str">
-        <x:v>Not yet agreed</x:v>
+        <x:v>8 October 2026</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="42" customHeight="1">
@@ -6127,7 +6127,7 @@
         <x:v>Verification result</x:v>
       </x:c>
       <x:c r="B131" s="7" t="str">
-        <x:v>Pending — no entitlement or resolution conclusion</x:v>
+        <x:v>Verified: net £180 agrees with 120 pallet-days at £1.50. The billing correction is closed for this line.</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="42" customHeight="1">
@@ -6135,7 +6135,7 @@
         <x:v>Decision / resources needed</x:v>
       </x:c>
       <x:c r="B132" s="7" t="str">
-        <x:v>Resolve any outstanding commercial interpretation and present it alongside the service and storage evidence.</x:v>
+        <x:v>Accept the verified credit for this line. Commercial lead checks contract timetable/options while the director awaits service and quality evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="42" customHeight="1">
@@ -6143,7 +6143,7 @@
         <x:v>Decision owner</x:v>
       </x:c>
       <x:c r="B133" s="7" t="str">
-        <x:v>Commercial/finance authority to be established; logistics director for renewal</x:v>
+        <x:v>Commercial lead for the credit; logistics director for the separate final renewal decision.</x:v>
       </x:c>
     </x:row>
     <x:row r="134" ht="30" customHeight="1">
@@ -6155,7 +6155,7 @@
         <x:v>Management note</x:v>
       </x:c>
       <x:c r="B135" s="7" t="str">
-        <x:v>The director's renewal decision remains open. A service finding does not settle storage acceptability, provider qualification or invoice entitlement.</x:v>
+        <x:v>As at 8 October, the director awaits the quality assessment due 9 October and service plan due 10 October. Commercial lead checks contract timetable/options. The verified £60 credit does not settle renewal or product acceptability.</x:v>
       </x:c>
     </x:row>
     <x:row r="136" ht="30" customHeight="1">

</xml_diff>